<commit_message>
test agent updated, batching added
</commit_message>
<xml_diff>
--- a/output_req.xlsx
+++ b/output_req.xlsx
@@ -451,7 +451,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[2, 3, 4, 5, 8, 9, 11, 19, 22, 26]</t>
+          <t>[2, 3, 4, 5, 8, 9, 22, 26, 27, 31]</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -466,7 +466,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[1, 9]</t>
+          <t>[1, 5, 9, 31]</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Household Composition and Eligibility Assessment</t>
+          <t>Household Composition Management</t>
         </is>
       </c>
     </row>
@@ -511,12 +511,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>[1, 11, 22]</t>
+          <t>[1, 2, 11, 12, 22]</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Application Completeness Checking</t>
+          <t>Application Incompleteness Detection</t>
         </is>
       </c>
     </row>
@@ -526,12 +526,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[7, 23, 30, 32, 34, 36]</t>
+          <t>[7, 23, 25, 34]</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Case Management Dashboard—Eligibility Tracking</t>
+          <t>Eligibility Status Dashboard</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Eligibility Expiration Alerts &amp; Redetermination</t>
+          <t>Eligibility Expiry Alert System</t>
         </is>
       </c>
     </row>
@@ -556,12 +556,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[1, 12, 17, 19, 21, 24, 29, 39]</t>
+          <t>[1, 11, 12, 17, 21, 24, 29, 39]</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Document Management—Upload Capability</t>
+          <t>Document Upload Management</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Applicant Search and Duplicate Prevention</t>
+          <t>Applicant Search &amp; De-duplication</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Case Assignment and Workload Balancing</t>
+          <t>Case Assignment and Workload Management</t>
         </is>
       </c>
     </row>
@@ -601,12 +601,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>[5, 12, 17]</t>
+          <t>[5, 8, 12, 17, 21]</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Document Request and Secure Communication</t>
+          <t>Document Request and Notification</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>[8, 11, 17, 21]</t>
+          <t>[5, 8, 11, 17, 21]</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -631,12 +631,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>[8, 29]</t>
+          <t>[8, 21, 29]</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Document Privacy Redaction Tools</t>
+          <t>Document Redaction/Privacy Management</t>
         </is>
       </c>
     </row>
@@ -646,12 +646,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>[15, 20, 25]</t>
+          <t>[6, 20]</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Case Communication Log</t>
+          <t>Client Communication Log</t>
         </is>
       </c>
     </row>
@@ -661,12 +661,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>[14]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dual Eligibility &amp; Inter-agency Case Coordination</t>
+          <t>Inter-agency Case Coordination</t>
         </is>
       </c>
     </row>
@@ -676,12 +676,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>[1, 35]</t>
+          <t>[3, 4, 6, 25, 32, 35]</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Eligibility Findings Reporting</t>
+          <t>Eligibility Summary &amp; Reporting</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Real-time Alerts for Document Uploads</t>
+          <t>Document Upload Notification</t>
         </is>
       </c>
     </row>
@@ -706,7 +706,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>[10, 32, 40]</t>
+          <t>[6, 10, 32, 40]</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -721,12 +721,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>[1, 8, 26]</t>
+          <t>[5, 8, 21, 26]</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Printable Document Checklist</t>
+          <t>Document Checklist Printing</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>[8, 12]</t>
+          <t>[8, 11, 12, 13, 19]</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AI-assisted Field Completion Suggestions</t>
+          <t>AI Application Field Completion Suggestions</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>[6, 32]</t>
+          <t>[6, 25, 32]</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -811,12 +811,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>[14]</t>
+          <t>[6, 16, 23]</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Denial Analytics &amp; Reporting</t>
+          <t>Eligibility Denial Analytics</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Pre-fill Application Data</t>
+          <t>Application Data Pre-fill</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>[4]</t>
+          <t>[4, 1]</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -876,7 +876,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Document Preview Functionality</t>
+          <t>Document Preview Before Upload</t>
         </is>
       </c>
     </row>
@@ -886,12 +886,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>[6]</t>
+          <t>[32, 23]</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Case Data Export (CSV/Excel)</t>
+          <t>Case Data Export</t>
         </is>
       </c>
     </row>
@@ -901,12 +901,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>[9]</t>
+          <t>[1, 2, 9]</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Duplicate Application Detection</t>
+          <t>Duplicate Application Detection &amp; Merge</t>
         </is>
       </c>
     </row>
@@ -916,12 +916,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>[6, 18, 23]</t>
+          <t>[16, 18, 23, 30]</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Case Activity Monthly Reporting</t>
+          <t>Case Activity &amp; Team Performance Reporting</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Overdue Redetermination Tracking</t>
+          <t>Redetermination Tracking</t>
         </is>
       </c>
     </row>
@@ -966,7 +966,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Printable Case Note Summary</t>
+          <t>Case Note Summary Printing</t>
         </is>
       </c>
     </row>
@@ -976,12 +976,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>[6]</t>
+          <t>[6, 40]</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Inactivity Alerts for Follow-Up</t>
+          <t>Inactive Case Alerts</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Escalated Case Trend Reporting</t>
+          <t>Escalated Case Metrics</t>
         </is>
       </c>
     </row>
@@ -1036,12 +1036,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>[10, 18]</t>
+          <t>[10, 18, 36]</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Overloaded Caseworker Alert &amp; Reassignment</t>
+          <t>Caseworker Overload Alert &amp; Reassignment</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agent can successfully call query function
</commit_message>
<xml_diff>
--- a/output_req.xlsx
+++ b/output_req.xlsx
@@ -451,12 +451,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[2, 3, 4, 5, 8, 9, 22, 26, 27, 31]</t>
+          <t>[2, 3, 4, 5, 8, 9, 11, 12, 19, 22, 26, 31]</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Medicaid Application Intake Module</t>
+          <t>Medicaid Application Intake (Case Worker) – Entering new applicant and case creation</t>
         </is>
       </c>
     </row>
@@ -466,12 +466,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[1, 5, 9, 31]</t>
+          <t>[1, 3, 33]</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Applicant Identity Verification</t>
+          <t>Identity Verification (Case Worker) – Integration with external government ID services</t>
         </is>
       </c>
     </row>
@@ -481,12 +481,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>[1, 37]</t>
+          <t>[1, 2, 37]</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Income Eligibility Verification</t>
+          <t>Income Verification (Case Worker) – Checking eligibility through wage and data verification</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Household Composition Management</t>
+          <t>Household Composition Management (Case Worker) – Recording family members for eligibility</t>
         </is>
       </c>
     </row>
@@ -511,12 +511,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>[1, 2, 11, 12, 22]</t>
+          <t>[1, 12, 11, 22]</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Application Incompleteness Detection</t>
+          <t>Application Completeness Monitoring (Case Worker) – Flagging missing information</t>
         </is>
       </c>
     </row>
@@ -526,12 +526,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[7, 23, 25, 34]</t>
+          <t>[7, 23, 25, 30, 32, 34, 36]</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eligibility Status Dashboard</t>
+          <t>Eligibility Status Dashboard (Case Manager) – Viewing clients’ status and renewals</t>
         </is>
       </c>
     </row>
@@ -541,12 +541,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>[6, 34]</t>
+          <t>[6, 34, 36]</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Eligibility Expiry Alert System</t>
+          <t>Eligibility Expiration Alerts (Case Manager) – Notification before eligibility lapses</t>
         </is>
       </c>
     </row>
@@ -556,12 +556,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[1, 11, 12, 17, 21, 24, 29, 39]</t>
+          <t>[1, 11, 12, 13, 17, 21, 24, 29, 39]</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Document Upload Management</t>
+          <t>Document Upload (Case Worker) – Maintaining supporting files and attachments</t>
         </is>
       </c>
     </row>
@@ -571,12 +571,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>[1, 2, 31]</t>
+          <t>[1, 31]</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Applicant Search &amp; De-duplication</t>
+          <t>Duplicate Application Prevention (Case Worker) – Searching applicants to avoid redundancy</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Case Assignment and Workload Management</t>
+          <t>Case Assignment (Case Manager) – Assign and balance caseloads among team</t>
         </is>
       </c>
     </row>
@@ -601,12 +601,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>[5, 8, 12, 17, 21]</t>
+          <t>[1, 5, 8, 12, 17]</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Document Request and Notification</t>
+          <t>Document Request &amp; Communication (Case Worker) – Requesting missing info from applicants</t>
         </is>
       </c>
     </row>
@@ -616,12 +616,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>[5, 8, 11, 17, 21]</t>
+          <t>[5, 8, 11, 17]</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Document Submission Tracking</t>
+          <t>Document Submission Tracking (Case Worker) – Monitoring pending and submitted files</t>
         </is>
       </c>
     </row>
@@ -631,12 +631,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>[8, 21, 29]</t>
+          <t>[8]</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Document Redaction/Privacy Management</t>
+          <t>Sensitive Data Redaction (Case Worker) – Redacting private info in uploaded documents</t>
         </is>
       </c>
     </row>
@@ -646,12 +646,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>[6, 20]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Client Communication Log</t>
+          <t>Client Communication Log (Case Manager) – Viewing email, call, and message history</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Inter-agency Case Coordination</t>
+          <t>Inter-Agency Coordination (Case Manager) – Supporting dual-eligibility and information sharing</t>
         </is>
       </c>
     </row>
@@ -676,12 +676,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>[3, 4, 6, 25, 32, 35]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Eligibility Summary &amp; Reporting</t>
+          <t>Eligibility Findings Reporting (Case Worker) – Auto-generating summary reports</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Document Upload Notification</t>
+          <t>Document Upload Alerts (Case Worker) – Notifying when documents are submitted</t>
         </is>
       </c>
     </row>
@@ -706,12 +706,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>[6, 10, 32, 40]</t>
+          <t>[32, 40]</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Case Time Tracking</t>
+          <t>Case Time Tracking (Case Manager) – Logging work time for reporting</t>
         </is>
       </c>
     </row>
@@ -721,12 +721,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>[5, 8, 21, 26]</t>
+          <t>[1, 5, 26]</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Document Checklist Printing</t>
+          <t>Printable Document Checklist (Case Worker) – Providing clients with required document lists</t>
         </is>
       </c>
     </row>
@@ -736,12 +736,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>[14, 38]</t>
+          <t>[38]</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Case Escalation Workflow</t>
+          <t>Case Escalation (Case Manager) – Urgent case workflow and supervisor notification</t>
         </is>
       </c>
     </row>
@@ -751,12 +751,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>[8, 11, 12, 13, 19]</t>
+          <t>[8]</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Automated Document Validation</t>
+          <t>Document Auto-Validation (Case Worker) – Automated checks on uploaded documents</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AI Application Field Completion Suggestions</t>
+          <t>Application Field Completion Suggestions (Case Worker) – Assisting in data entry</t>
         </is>
       </c>
     </row>
@@ -781,12 +781,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>[6, 25, 32]</t>
+          <t>[6]</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Eligibility Status Filtering</t>
+          <t>Client Eligibility Filtering (Case Manager) – Sort/filter clients by eligibility status</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Bulk Document Upload</t>
+          <t>Bulk Document Upload (Case Worker) – Uploading files for multiple cases simultaneously</t>
         </is>
       </c>
     </row>
@@ -811,12 +811,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>[6, 16, 23]</t>
+          <t>[6]</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Eligibility Denial Analytics</t>
+          <t>Denial Trend Analytics (Case Manager) – Viewing trends in eligibility denials</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Application Data Pre-fill</t>
+          <t>Data Pre-fill from Previous Cases (Case Worker) – Reducing repeated manual entry</t>
         </is>
       </c>
     </row>
@@ -841,12 +841,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>[4, 1]</t>
+          <t>[4]</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Household Data Conflict Alerts</t>
+          <t>Household Data Conflict Alerts (Case Worker) – Resolving household info discrepancies</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Case Assignment by Language Preference</t>
+          <t>Language-Based Case Assignment (Case Manager) – Matching client and caseworker languages</t>
         </is>
       </c>
     </row>
@@ -871,12 +871,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>[8, 13]</t>
+          <t>[8]</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Document Preview Before Upload</t>
+          <t>Document Preview Before Upload (Case Worker) – Confirming accuracy of uploads</t>
         </is>
       </c>
     </row>
@@ -886,12 +886,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>[32, 23]</t>
+          <t>[6]</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Case Data Export</t>
+          <t>Case Data Export (Case Manager) – CSV/Excel download for offline analysis</t>
         </is>
       </c>
     </row>
@@ -901,12 +901,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>[1, 2, 9]</t>
+          <t>[1, 9]</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Duplicate Application Detection &amp; Merge</t>
+          <t>Duplicate Application Alerts (Case Worker) – Detecting and merging duplicate entries</t>
         </is>
       </c>
     </row>
@@ -916,12 +916,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>[16, 18, 23, 30]</t>
+          <t>[6, 18]</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Case Activity &amp; Team Performance Reporting</t>
+          <t>Case Activity Reporting (Case Manager) – Generating monthly and filtered reports</t>
         </is>
       </c>
     </row>
@@ -931,12 +931,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[2]</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Eligibility Rule Change Notification</t>
+          <t>Eligibility Policy Change Alerts (Case Worker) – Informing about rule updates</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Redetermination Tracking</t>
+          <t>Overdue Redetermination Tracking (Case Manager) – Monitoring overdue eligibility cases</t>
         </is>
       </c>
     </row>
@@ -961,12 +961,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>[16]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Case Note Summary Printing</t>
+          <t>Printable Case Note Summaries (Case Worker) – Produce physical copies for files</t>
         </is>
       </c>
     </row>
@@ -976,12 +976,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>[6, 40]</t>
+          <t>[6, 7]</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Inactive Case Alerts</t>
+          <t>Inactive Case Alerts (Case Manager) – Notifying on inactivity for follow-up</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Conflicting Income Data Alerts</t>
+          <t>Conflicting Income Alerts (Case Worker) – Investigate inconsistencies in income data</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Escalated Case Metrics</t>
+          <t>Escalation Metrics (Case Manager) – Tracking number and trends of escalated cases</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>After-Hours Document Upload Alerts</t>
+          <t>After-Hours Upload Alerts (Case Worker) – Prioritizing late document reviews</t>
         </is>
       </c>
     </row>
@@ -1036,12 +1036,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>[10, 18, 36]</t>
+          <t>[10, 18]</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Caseworker Overload Alert &amp; Reassignment</t>
+          <t>Caseworker Overload Alerts (Case Manager) – Monitoring and reallocating caseload</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Successfully integrated database with requirement agent
</commit_message>
<xml_diff>
--- a/output_req.xlsx
+++ b/output_req.xlsx
@@ -447,601 +447,601 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>22895813</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[2, 3, 4, 5, 8, 9, 11, 12, 19, 22, 26, 31]</t>
+          <t>[22895823, 22895830, 22895814, 22895841, 22895832]</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Medicaid Application Intake (Case Worker) – Entering new applicant and case creation</t>
+          <t>Eligibility Management / Status Viewing</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>22895831</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[1, 3, 33]</t>
+          <t>[22895815, 22895836, 22895828, 22895820]</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Identity Verification (Case Worker) – Integration with external government ID services</t>
+          <t>Document Management / Bulk Upload</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>22895823</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>[1, 2, 37]</t>
+          <t>[22895813, 22895832, 22895839]</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Income Verification (Case Worker) – Checking eligibility through wage and data verification</t>
+          <t>Reporting / Eligibility Summary</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>22895836</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[1, 27]</t>
+          <t>[22895831, 22895815, 22895828]</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Household Composition Management (Case Worker) – Recording family members for eligibility</t>
+          <t>Document Management / Document Preview</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>22895834</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>[1, 12, 11, 22]</t>
+          <t>[22895811, 22895844, 22895816]</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Application Completeness Monitoring (Case Worker) – Flagging missing information</t>
+          <t>Data Quality / Household Data Alerts</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>22895846</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[7, 23, 25, 30, 32, 34, 36]</t>
+          <t>[22895824, 22895819]</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eligibility Status Dashboard (Case Manager) – Viewing clients’ status and renewals</t>
+          <t>Alerts / Document Upload (After Hours)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>22895824</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>[6, 34, 36]</t>
+          <t>[22895846, 22895819]</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Eligibility Expiration Alerts (Case Manager) – Notification before eligibility lapses</t>
+          <t>Alerts / Document Upload Notification</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
+        <v>22895829</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[1, 11, 12, 13, 17, 21, 24, 29, 39]</t>
+          <t>[22895812, 22895833]</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Document Upload (Case Worker) – Maintaining supporting files and attachments</t>
+          <t>Application Assistance / Field Suggestions</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
+        <v>22895811</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>[1, 31]</t>
+          <t>[22895834, 22895810]</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Duplicate Application Prevention (Case Worker) – Searching applicants to avoid redundancy</t>
+          <t>Household Management / Composition Recording</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10</v>
+        <v>22895820</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>[28, 40]</t>
+          <t>[22895815, 22895831]</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Case Assignment (Case Manager) – Assign and balance caseloads among team</t>
+          <t>Document Management / Redaction</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11</v>
+        <v>22895816</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>[1, 5, 8, 12, 17]</t>
+          <t>[22895834, 22895838, 22895808]</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Document Request &amp; Communication (Case Worker) – Requesting missing info from applicants</t>
+          <t>Applicant Management / Search and Deduplication</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>12</v>
+        <v>22895818</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>[5, 8, 11, 17]</t>
+          <t>[22895819, 22895824, 22895826]</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Document Submission Tracking (Case Worker) – Monitoring pending and submitted files</t>
+          <t>Applicant Communication / Document Requests</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>13</v>
+        <v>22895815</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>[8]</t>
+          <t>[22895831, 22895836, 22895820]</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Sensitive Data Redaction (Case Worker) – Redacting private info in uploaded documents</t>
+          <t>Document Management / Uploading</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>14</v>
+        <v>22895809</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[22895810]</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Client Communication Log (Case Manager) – Viewing email, call, and message history</t>
+          <t>Identity Management / Applicant Verification</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>22895835</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[22895817, 22895847]</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Inter-Agency Coordination (Case Manager) – Supporting dual-eligibility and information sharing</t>
+          <t>Case Assignment / Language Preference</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>16</v>
+        <v>22895817</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[22895835, 22895847, 22895825, 22895827]</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Eligibility Findings Reporting (Case Worker) – Auto-generating summary reports</t>
+          <t>Case Assignment / Workload Balancing</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>17</v>
+        <v>22895822</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>[8, 11, 12, 39]</t>
+          <t>[22895813, 22895830]</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Document Upload Alerts (Case Worker) – Notifying when documents are submitted</t>
+          <t>Cross-Agency Coordination / Dual Eligibility</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>18</v>
+        <v>22895827</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>[32, 40]</t>
+          <t>[22895817, 22895845]</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Case Time Tracking (Case Manager) – Logging work time for reporting</t>
+          <t>Case Escalation / Supervisor Notification</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>19</v>
+        <v>22895837</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>[1, 5, 26]</t>
+          <t>[22895825, 22895839]</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Printable Document Checklist (Case Worker) – Providing clients with required document lists</t>
+          <t>Reporting / Data Export (Excel)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>20</v>
+        <v>22895830</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>[38]</t>
+          <t>[22895813, 22895822]</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Case Escalation (Case Manager) – Urgent case workflow and supervisor notification</t>
+          <t>Case Filtering / Eligibility Status</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>21</v>
+        <v>22895843</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>[8]</t>
+          <t>[22895841, 22895814]</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Document Auto-Validation (Case Worker) – Automated checks on uploaded documents</t>
+          <t>Alerts / Inactive Case Notification</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>22</v>
+        <v>22895847</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>[1, 5]</t>
+          <t>[22895817, 22895835]</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Application Field Completion Suggestions (Case Worker) – Assisting in data entry</t>
+          <t>Alerts / Caseworker Overload</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>23</v>
+        <v>22895814</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>[6]</t>
+          <t>[22895813, 22895843, 22895841]</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Client Eligibility Filtering (Case Manager) – Sort/filter clients by eligibility status</t>
+          <t>Alerts / Eligibility Expiry</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>24</v>
+        <v>22895841</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>[8]</t>
+          <t>[22895814, 22895843, 22895813]</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Bulk Document Upload (Case Worker) – Uploading files for multiple cases simultaneously</t>
+          <t>Compliance / Redetermination Tracking</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>25</v>
+        <v>22895845</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>[6]</t>
+          <t>[22895827]</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Denial Trend Analytics (Case Manager) – Viewing trends in eligibility denials</t>
+          <t>Case Tracking / Escalated Case Reporting</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>26</v>
+        <v>22895825</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>[1, 19]</t>
+          <t>[22895817, 22895837]</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Data Pre-fill from Previous Cases (Case Worker) – Reducing repeated manual entry</t>
+          <t>Case Metrics / Time Tracking</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>27</v>
+        <v>22895832</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>[4]</t>
+          <t>[22895813, 22895823]</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Household Data Conflict Alerts (Case Worker) – Resolving household info discrepancies</t>
+          <t>Reporting / Denial Trends</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>28</v>
+        <v>22895828</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>[10]</t>
+          <t>[22895831, 22895836]</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Language-Based Case Assignment (Case Manager) – Matching client and caseworker languages</t>
+          <t>Document Validation / Auto-Validation</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>29</v>
+        <v>22895810</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>[8]</t>
+          <t>[22895811, 22895809, 22895813]</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Document Preview Before Upload (Case Worker) – Confirming accuracy of uploads</t>
+          <t>Eligibility Management / Income Check</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>30</v>
+        <v>22895812</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>[6]</t>
+          <t>[22895829, 22895818]</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Case Data Export (Case Manager) – CSV/Excel download for offline analysis</t>
+          <t>Application Management / Incomplete Flag</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>31</v>
+        <v>22895808</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>[1, 9]</t>
+          <t>[22895816]</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Duplicate Application Alerts (Case Worker) – Detecting and merging duplicate entries</t>
+          <t>Applicant Intake / Medicaid Intake</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>32</v>
+        <v>22895826</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>[6, 18]</t>
+          <t>[22895818, 22895842]</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Case Activity Reporting (Case Manager) – Generating monthly and filtered reports</t>
+          <t>Document Management / Checklist Printing</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>33</v>
+        <v>22895842</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>[2]</t>
+          <t>[22895826]</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Eligibility Policy Change Alerts (Case Worker) – Informing about rule updates</t>
+          <t>Reporting / Case Notes Printing</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>34</v>
+        <v>22895838</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>[6, 7]</t>
+          <t>[22895816, 22895833]</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Overdue Redetermination Tracking (Case Manager) – Monitoring overdue eligibility cases</t>
+          <t>Applicant Management / Duplicate Alerts</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>35</v>
+        <v>22895844</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[22895834, 22895810]</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Printable Case Note Summaries (Case Worker) – Produce physical copies for files</t>
+          <t>Alerts / Conflicting Income</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>36</v>
+        <v>22895840</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>[6, 7]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Inactive Case Alerts (Case Manager) – Notifying on inactivity for follow-up</t>
+          <t>Compliance / Eligibility Rule Changes</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>37</v>
+        <v>22895819</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>[3]</t>
+          <t>[22895818, 22895824, 22895846]</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Conflicting Income Alerts (Case Worker) – Investigate inconsistencies in income data</t>
+          <t>Document Management / Submission Tracking</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>38</v>
+        <v>22895839</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>[20]</t>
+          <t>[22895837, 22895823]</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Escalation Metrics (Case Manager) – Tracking number and trends of escalated cases</t>
+          <t>Reporting / Monthly Case Activity</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>39</v>
+        <v>22895821</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>[8, 17]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>After-Hours Upload Alerts (Case Worker) – Prioritizing late document reviews</t>
+          <t>Case Management / Communication Logs</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>40</v>
+        <v>22895833</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>[10, 18]</t>
+          <t>[22895829, 22895838]</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Caseworker Overload Alerts (Case Manager) – Monitoring and reallocating caseload</t>
+          <t>Application Management / Data Prefill</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Neo4j Knowledge Graph Boilerplate Code
</commit_message>
<xml_diff>
--- a/output_req.xlsx
+++ b/output_req.xlsx
@@ -447,397 +447,397 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>22895831</v>
+        <v>22895834</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[22895815, 22895836, 22895828, 22895820, 22895819]</t>
+          <t>[22895844, 22895838]</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bulk document upload module for case management</t>
+          <t>Data Validation &amp; Alerting - Conflicting Household Data</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>22895823</v>
+        <v>22895846</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[22895813, 22895832, 22895839]</t>
+          <t>[22895824]</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Eligibility summary reporting feature</t>
+          <t>Alerting - Document Uploads Outside Business Hours</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>22895836</v>
+        <v>22895829</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>[22895831, 22895815, 22895828, 22895820]</t>
+          <t>[22895833, 22895812]</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Document upload preview feature</t>
+          <t>Application Completeness/Suggestion Engine</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>22895834</v>
+        <v>22895816</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[22895811, 22895844]</t>
+          <t>[22895838, 22895809]</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Household data validation and alerting system</t>
+          <t>Applicant Search &amp; Duplicate Prevention</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>22895846</v>
+        <v>22895835</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>[22895824, 22895819]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Document upload alerting system for after-hours uploads</t>
+          <t>Case Assignment - Language Preference</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>22895829</v>
+        <v>22895827</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[22895812, 22895833, 22895808]</t>
+          <t>[22895845, 22895847]</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Application field validation and suggestions</t>
+          <t>Case Escalation/Workflow Management</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>22895816</v>
+        <v>22895843</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>[22895838, 22895808]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Applicant search and duplicate detection</t>
+          <t>Alerting - Inactive Case Notification</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>22895818</v>
+        <v>22895841</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[22895819, 22895815, 22895824]</t>
+          <t>[22895814]</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Document request and applicant upload coordination</t>
+          <t>Compliance Tracking - Redeterminations</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>22895815</v>
+        <v>22895845</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>[22895831, 22895836, 22895818, 22895819, 22895820, 22895828]</t>
+          <t>[22895827]</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Case document upload functionality</t>
+          <t>Case Escalation Reporting</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>22895809</v>
+        <v>22895813</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>[22895808, 22895810]</t>
+          <t>[22895830]</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Applicant identity verification module</t>
+          <t>Eligibility Status Viewing</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>22895835</v>
+        <v>22895832</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>[22895817, 22895827, 22895847]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Case assignment based on language preference</t>
+          <t>Analytics - Eligibility Denial Trends</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>22895817</v>
+        <v>22895831</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>[22895835, 22895827, 22895847, 22895825]</t>
+          <t>[22895836, 22895828, 22895815]</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Case workload-based assignment</t>
+          <t>Document Uploads - Bulk Upload</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>22895827</v>
+        <v>22895810</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>[22895835, 22895817, 22895845]</t>
+          <t>[22895844, 22895811]</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Urgent case escalation</t>
+          <t>Eligibility Calculation - Income Verification</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>22895837</v>
+        <v>22895823</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[22895813, 22895839]</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Case data export to Excel</t>
+          <t>Reporting - Eligibility Summary</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>22895843</v>
+        <v>22895836</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>[22895841, 22895808, 22895813]</t>
+          <t>[22895831, 22895815]</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Inactive case alert system</t>
+          <t>Document Uploads - Preview Feature</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>22895847</v>
+        <v>22895826</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>[22895835, 22895817]</t>
+          <t>[22895815, 22895812]</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Overloaded caseworker alert system</t>
+          <t>Document Checklist/Print Function</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>22895814</v>
+        <v>22895842</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>[22895841, 22895813]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Eligibility expiration alerting and redetermination initiation</t>
+          <t>Case Notes - Printing</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>22895841</v>
+        <v>22895838</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>[22895814, 22895843]</t>
+          <t>[22895816, 22895834]</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Overdue redetermination tracking</t>
+          <t>Applicant Duplicate Detection &amp; Alerting</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>22895845</v>
+        <v>22895824</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>[22895827]</t>
+          <t>[22895846, 22895819]</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Tracking and reporting on escalated cases</t>
+          <t>Alerting - Client Document Upload</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>22895825</v>
+        <v>22895811</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>[22895817]</t>
+          <t>[22895810]</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Case time tracking and reporting</t>
+          <t>Eligibility Calculation - Household Composition</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>22895813</v>
+        <v>22895820</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>[22895814, 22895823, 22895830, 22895843]</t>
+          <t>[22895836, 22895828]</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Client eligibility status overview</t>
+          <t>Document Handling - Redaction</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>22895832</v>
+        <v>22895818</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>[22895823, 22895813]</t>
+          <t>[22895815, 22895819]</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Eligibility denial trend analysis</t>
+          <t>Document Request/Communication with Applicants</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>22895828</v>
+        <v>22895819</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>[22895831, 22895815, 22895836]</t>
+          <t>[22895818, 22895824]</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Automated document validation</t>
+          <t>Document Submission Tracking</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>22895810</v>
+        <v>22895815</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>[22895809, 22895808]</t>
+          <t>[22895836, 22895831, 22895826, 22895818]</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Income eligibility checking</t>
+          <t>Document Uploads - Case Attachments</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>22895812</v>
+        <v>22895809</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>[22895829, 22895833]</t>
+          <t>[22895816]</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Incomplete application flagging</t>
+          <t>Identity Verification</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>22895808</v>
+        <v>22895817</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>[22895809, 22895810, 22895816, 22895812, 22895843]</t>
+          <t>[22895825, 22895847]</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>New Medicaid application intake</t>
+          <t>Case Assignment - Workload Balancing</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>22895826</v>
+        <v>22895822</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -846,202 +846,202 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Printing required documents checklist</t>
+          <t>Eligibility Coordination - Dual Agency</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>22895842</v>
+        <v>22895837</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[22895839]</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Printing case notes summary</t>
+          <t>Data Export - Excel</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>22895838</v>
+        <v>22895830</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>[22895816]</t>
+          <t>[22895813]</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Duplicate application alert and merge</t>
+          <t>Client Filtering - Eligibility Status</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>22895844</v>
+        <v>22895847</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>[22895834]</t>
+          <t>[22895817, 22895827]</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Conflicting income data alerts</t>
+          <t>Alerting - Caseworker Workload</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>22895824</v>
+        <v>22895814</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>[22895846, 22895818, 22895819]</t>
+          <t>[22895841]</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Client document upload notification</t>
+          <t>Alerting - Eligibility Expiry</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>22895840</v>
+        <v>22895825</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[22895817]</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Eligibility rules change alerts</t>
+          <t>Workload Tracking &amp; Reporting</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>22895811</v>
+        <v>22895828</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>[22895834]</t>
+          <t>[22895831, 22895820]</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Household composition recording</t>
+          <t>Document Handling - Auto-validation</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>22895820</v>
+        <v>22895812</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>[22895831, 22895815, 22895836]</t>
+          <t>[22895829, 22895826]</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Redaction of sensitive document information</t>
+          <t>Application Completeness/Flagging</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>22895819</v>
+        <v>22895808</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>[22895824, 22895818, 22895815, 22895846, 22895831]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Document submission status tracking</t>
+          <t>Medicaid Application Intake</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>22895822</v>
+        <v>22895844</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[22895810, 22895834]</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Inter-agency coordination for dual eligibility</t>
+          <t>Alerting - Conflicting Income Data</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>22895830</v>
+        <v>22895840</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>[22895813]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Client filtering by eligibility status</t>
+          <t>Alerting - Eligibility Rule Changes</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>22895833</v>
+        <v>22895839</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>[22895829, 22895812]</t>
+          <t>[22895837, 22895823]</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Pre-filling application data</t>
+          <t>Reporting - Monthly Case Activity</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>22895839</v>
+        <v>22895821</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>[22895823]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Monthly case activity reporting</t>
+          <t>Case Communication Logs</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>22895821</v>
+        <v>22895833</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[22895829]</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Client communication log viewing</t>
+          <t>Application Data Prefilling</t>
         </is>
       </c>
     </row>

</xml_diff>